<commit_message>
feat(ui): implement executive dashboard foundation
</commit_message>
<xml_diff>
--- a/data/workbook/Requests.xlsx
+++ b/data/workbook/Requests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eoh.sharepoint.com/sites/ISETSSolutions/Shared Documents/Solution Requests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Christopher.Young\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{244155B2-1582-4B7D-971D-F4FA5652BFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B9E8A61-9D92-4827-B705-402F71451ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{35526BAD-6773-4E2C-BDFB-6CE53E6E1FA5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{35526BAD-6773-4E2C-BDFB-6CE53E6E1FA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Technical Assistance" sheetId="8" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="253">
   <si>
     <t>Customer</t>
   </si>
@@ -796,6 +796,12 @@
   </si>
   <si>
     <t>Floyd</t>
+  </si>
+  <si>
+    <t>Dell R470 Config</t>
+  </si>
+  <si>
+    <t>Entry Level Single CPU for Dean</t>
   </si>
 </sst>
 </file>
@@ -805,7 +811,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1257,18 +1263,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C8B9304-19BA-4974-A075-F6081784C26F}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="8" customWidth="1"/>
-    <col min="4" max="4" width="43.28515625" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="43.33203125" customWidth="1"/>
     <col min="5" max="5" width="33" customWidth="1"/>
-    <col min="6" max="6" width="68.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" customWidth="1"/>
+    <col min="6" max="6" width="68.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1291,7 +1297,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -1314,7 +1320,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
@@ -1337,7 +1343,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
@@ -1360,7 +1366,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
@@ -1381,7 +1387,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>26</v>
       </c>
@@ -1404,7 +1410,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>30</v>
       </c>
@@ -1427,7 +1433,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
@@ -1450,7 +1456,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -1473,7 +1479,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
@@ -1496,7 +1502,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1519,7 +1525,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -1539,7 +1545,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -1562,7 +1568,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>51</v>
       </c>
@@ -1585,7 +1591,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -1608,7 +1614,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>56</v>
       </c>
@@ -1631,7 +1637,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>56</v>
       </c>
@@ -1654,7 +1660,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1677,7 +1683,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>63</v>
       </c>
@@ -1700,7 +1706,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>67</v>
       </c>
@@ -1723,7 +1729,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>70</v>
       </c>
@@ -1746,7 +1752,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -1766,7 +1772,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1789,7 +1795,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -1809,7 +1815,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>80</v>
       </c>
@@ -1832,7 +1838,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>80</v>
       </c>
@@ -1888,19 +1894,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87F45B4A-8A03-487F-84B4-9E8F403D3277}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" style="3" customWidth="1"/>
     <col min="2" max="2" width="16" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="25.28515625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="3"/>
+    <col min="3" max="3" width="14.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="25.33203125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1923,7 +1929,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>85</v>
       </c>
@@ -1946,7 +1952,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="28.9">
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>88</v>
       </c>
@@ -1969,7 +1975,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29.25">
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>91</v>
       </c>
@@ -2020,21 +2026,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F1D1FF-D0D7-48FE-B9BC-9DE425333CC3}">
-  <dimension ref="A1:H54"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <dimension ref="A1:H55"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="46.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="43.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="8.85546875" style="3"/>
+    <col min="2" max="2" width="24.5546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" style="7" customWidth="1"/>
+    <col min="4" max="4" width="46.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="43.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.25" customHeight="1">
+    <row r="1" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2060,7 +2066,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="31.5" customHeight="1">
+    <row r="2" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>96</v>
       </c>
@@ -2086,7 +2092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.9">
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>100</v>
       </c>
@@ -2112,7 +2118,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>104</v>
       </c>
@@ -2138,7 +2144,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="43.5">
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>108</v>
       </c>
@@ -2164,7 +2170,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>111</v>
       </c>
@@ -2187,7 +2193,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>114</v>
       </c>
@@ -2213,7 +2219,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>117</v>
       </c>
@@ -2239,7 +2245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>120</v>
       </c>
@@ -2265,7 +2271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="28.9">
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>124</v>
       </c>
@@ -2288,7 +2294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>104</v>
       </c>
@@ -2314,7 +2320,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>129</v>
       </c>
@@ -2340,7 +2346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>41</v>
       </c>
@@ -2366,7 +2372,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>134</v>
       </c>
@@ -2392,7 +2398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>137</v>
       </c>
@@ -2418,7 +2424,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>104</v>
       </c>
@@ -2444,7 +2450,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>142</v>
       </c>
@@ -2470,7 +2476,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>145</v>
       </c>
@@ -2493,7 +2499,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="86.45">
+    <row r="19" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>148</v>
       </c>
@@ -2516,7 +2522,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="28.9">
+    <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>151</v>
       </c>
@@ -2539,7 +2545,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>154</v>
       </c>
@@ -2565,7 +2571,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="28.9">
+    <row r="22" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>157</v>
       </c>
@@ -2588,7 +2594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>160</v>
       </c>
@@ -2614,7 +2620,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="28.9">
+    <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>114</v>
       </c>
@@ -2640,7 +2646,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>142</v>
       </c>
@@ -2666,7 +2672,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="28.9">
+    <row r="26" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>137</v>
       </c>
@@ -2692,7 +2698,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>137</v>
       </c>
@@ -2718,7 +2724,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>171</v>
       </c>
@@ -2744,7 +2750,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>174</v>
       </c>
@@ -2770,7 +2776,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>129</v>
       </c>
@@ -2796,7 +2802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>179</v>
       </c>
@@ -2822,7 +2828,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>182</v>
       </c>
@@ -2848,7 +2854,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>70</v>
       </c>
@@ -2874,7 +2880,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>187</v>
       </c>
@@ -2894,7 +2900,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="28.9">
+    <row r="35" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>187</v>
       </c>
@@ -2920,7 +2926,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>154</v>
       </c>
@@ -2946,7 +2952,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>193</v>
       </c>
@@ -2972,7 +2978,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>196</v>
       </c>
@@ -2998,7 +3004,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="72">
+    <row r="39" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>196</v>
       </c>
@@ -3024,7 +3030,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>137</v>
       </c>
@@ -3050,7 +3056,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="29.25">
+    <row r="41" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
         <v>202</v>
       </c>
@@ -3073,7 +3079,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>205</v>
       </c>
@@ -3099,7 +3105,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>208</v>
       </c>
@@ -3125,7 +3131,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>210</v>
       </c>
@@ -3151,7 +3157,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="28.9">
+    <row r="45" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>212</v>
       </c>
@@ -3177,7 +3183,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>179</v>
       </c>
@@ -3203,7 +3209,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>216</v>
       </c>
@@ -3229,7 +3235,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>218</v>
       </c>
@@ -3255,7 +3261,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>88</v>
       </c>
@@ -3281,7 +3287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="43.5">
+    <row r="50" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>148</v>
       </c>
@@ -3304,7 +3310,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="28.9">
+    <row r="51" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>63</v>
       </c>
@@ -3330,7 +3336,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="28.9">
+    <row r="52" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>114</v>
       </c>
@@ -3356,7 +3362,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
         <v>218</v>
       </c>
@@ -3382,7 +3388,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="29.25">
+    <row r="54" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>231</v>
       </c>
@@ -3405,6 +3411,32 @@
         <v>94</v>
       </c>
       <c r="H54" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A55" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C55" s="7">
+        <v>46210</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H55" s="3" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3447,19 +3479,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57B2083C-1BC7-4AFC-8553-85C252212420}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.140625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="16" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="3"/>
+    <col min="3" max="3" width="15.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3482,7 +3514,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.9">
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>235</v>
       </c>
@@ -3505,7 +3537,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>124</v>
       </c>
@@ -3525,7 +3557,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="28.9">
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>145</v>
       </c>
@@ -3545,7 +3577,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="57.75">
+    <row r="5" spans="1:8" ht="58.8" x14ac:dyDescent="0.4">
       <c r="A5" s="10" t="s">
         <v>239</v>
       </c>
@@ -3565,7 +3597,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28.9">
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>241</v>
       </c>
@@ -3588,7 +3620,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.9">
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>47</v>
       </c>
@@ -3611,7 +3643,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="28.9">
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>244</v>
       </c>
@@ -3666,15 +3698,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1406E409-4030-437C-B85E-17AF60C85E1F}">
   <dimension ref="A2:F11"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.5703125" customWidth="1"/>
-    <col min="2" max="2" width="25.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="1" max="1" width="30.5546875" customWidth="1"/>
+    <col min="2" max="2" width="25.33203125" customWidth="1"/>
+    <col min="3" max="3" width="17.109375" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3691,7 +3723,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>8</v>
       </c>
@@ -3705,7 +3737,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>31</v>
       </c>
@@ -3719,7 +3751,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>48</v>
       </c>
@@ -3733,7 +3765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>138</v>
       </c>
@@ -3744,7 +3776,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>22</v>
       </c>
@@ -3752,7 +3784,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>14</v>
       </c>
@@ -3760,7 +3792,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>249</v>
       </c>
@@ -3768,7 +3800,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>250</v>
       </c>
@@ -3776,7 +3808,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D11" t="s">
         <v>38</v>
       </c>
@@ -3787,6 +3819,24 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <RequestID xmlns="b0f59d55-2e74-48ef-8b39-4628ff773f8d" xsi:nil="true"/>
+    <RequestID0 xmlns="b0f59d55-2e74-48ef-8b39-4628ff773f8d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100510EE39694FAC94EBA0A593490145454" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10d45ab09f7fe441f8e0bd96901553d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b0f59d55-2e74-48ef-8b39-4628ff773f8d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89f12b2ac4976b4ed6dab5d87063f5a0" ns2:_="">
     <xsd:import namespace="b0f59d55-2e74-48ef-8b39-4628ff773f8d"/>
@@ -3936,32 +3986,38 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <RequestID xmlns="b0f59d55-2e74-48ef-8b39-4628ff773f8d" xsi:nil="true"/>
-    <RequestID0 xmlns="b0f59d55-2e74-48ef-8b39-4628ff773f8d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97E7CDE3-4977-4329-9A03-B3356F207B17}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29201C4F-DEFF-4165-9A84-803DBA68C4E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B0FD9BF-5245-407E-87E5-6F8937C2E261}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B0FD9BF-5245-407E-87E5-6F8937C2E261}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b0f59d55-2e74-48ef-8b39-4628ff773f8d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29201C4F-DEFF-4165-9A84-803DBA68C4E4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97E7CDE3-4977-4329-9A03-B3356F207B17}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b0f59d55-2e74-48ef-8b39-4628ff773f8d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>